<commit_message>
User Upload excel enhancement
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/USERS-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/USERS-UPLOAD-TEMPLATE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\node proj\rest-api-nestjs\uploads\UPLOAD-TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429F1D3B-D2F8-47DE-90CA-C08547E20F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4C581F-02C6-42D1-9FC9-6A1457E11082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>Middle Name</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>SPA - NATIONWIDE ADMIN</t>
+  </si>
+  <si>
+    <t>Send Email Notif</t>
   </si>
 </sst>
 </file>
@@ -481,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE589B1-C7BA-44D4-9E29-919A5892AA9B}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -494,9 +497,10 @@
     <col min="8" max="8" width="16.109375" customWidth="1"/>
     <col min="9" max="9" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -530,8 +534,11 @@
       <c r="K1" s="5" t="s">
         <v>1</v>
       </c>
+      <c r="L1" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -559,8 +566,11 @@
       <c r="K2">
         <v>1</v>
       </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>12</v>
       </c>

</xml_diff>